<commit_message>
update wilcoxon & list
</commit_message>
<xml_diff>
--- a/liste.xlsx
+++ b/liste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sefa6\workspace\akademik\heuristic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65AB031C-AA35-4D08-8DD5-E35C09161AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91B8AAE-AA97-4EFC-AD87-AA776266FF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2DC5DBA8-4241-4F20-A30F-3D278B635267}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="329">
   <si>
     <t>S.N</t>
   </si>
@@ -1012,6 +1012,15 @@
   </si>
   <si>
     <t>LSHADE_CNEPSIN</t>
+  </si>
+  <si>
+    <t>LSHADE_SPACMA</t>
+  </si>
+  <si>
+    <t>Yusuf Kurt</t>
+  </si>
+  <si>
+    <t>Orkun Alp Alim</t>
   </si>
 </sst>
 </file>
@@ -1116,7 +1125,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1139,6 +1148,13 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1621,21 +1637,23 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
+      <c r="A9" s="9">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="4" t="s">
-        <v>9</v>
+      <c r="E9" s="9" t="s">
+        <v>327</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1735,21 +1753,21 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
+      <c r="A15" s="7">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="3"/>
-      <c r="F15" s="4" t="s">
-        <v>9</v>
+      <c r="E15" s="7"/>
+      <c r="F15" s="8" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -2029,21 +2047,23 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="3">
+      <c r="A30" s="10">
         <v>29</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="E30" s="3"/>
-      <c r="F30" s="4" t="s">
-        <v>9</v>
+      <c r="E30" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2955,24 +2975,25 @@
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" s="3">
+      <c r="A77" s="7">
         <v>76</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="B77" s="7" t="s">
         <v>280</v>
       </c>
-      <c r="C77" s="3" t="s">
+      <c r="C77" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="D77" s="3" t="s">
+      <c r="D77" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="E77" s="3"/>
-      <c r="F77" s="4" t="s">
-        <v>9</v>
+      <c r="E77" s="7"/>
+      <c r="F77" s="8" t="s">
+        <v>315</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>